<commit_message>
Atualização da Aula 12
</commit_message>
<xml_diff>
--- a/Aula_12/cadastro_aulo.xlsx
+++ b/Aula_12/cadastro_aulo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,13 +439,24 @@
           <t>João Paulo</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="B2" t="n">
+        <v>26</v>
       </c>
       <c r="C2" t="n">
         <v>1.78</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paloma Silva</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>